<commit_message>
Actualiza portafolio 2026-06-23 14:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46195.596250057875</v>
+        <v>46196.59712994213</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>231</v>
@@ -5477,7 +5477,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46195.596534745375</v>
+        <v>46196.601929791665</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>180</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-01 13:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -6132,7 +6132,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46203.16836844907</v>
+        <v>46204.19897075232</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>285</v>
@@ -6179,8 +6179,8 @@
       <c r="S80" s="6">
         <v>0</v>
       </c>
-      <c r="T80" s="12" t="s">
-        <v>117</v>
+      <c r="T80" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="U80" s="10" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-01 14:26 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -4515,7 +4515,7 @@
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46195.697430960645</v>
+        <v>46204.59404633102</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>198</v>
@@ -4625,9 +4625,11 @@
       <c r="B55" s="8">
         <v>46066.4884557176</v>
       </c>
-      <c r="C55" s="9"/>
+      <c r="C55" s="8">
+        <v>46204.594040208336</v>
+      </c>
       <c r="D55" s="8">
-        <v>46195.70018221065</v>
+        <v>46204.594042916666</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>206</v>
@@ -4690,7 +4692,7 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46195.69743164352</v>
+        <v>46204.59404793981</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>210</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 19:40 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -4515,7 +4515,7 @@
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46204.59404633102</v>
+        <v>46209.78872840278</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>198</v>
@@ -4629,7 +4629,7 @@
         <v>46204.594040208336</v>
       </c>
       <c r="D55" s="8">
-        <v>46204.594042916666</v>
+        <v>46209.811246377314</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>206</v>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46197.59005347222</v>
+        <v>46209.79759747685</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>230</v>
@@ -5359,9 +5359,11 @@
       <c r="B67" s="8">
         <v>46066.4884515625</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="8">
+        <v>46209.79758950231</v>
+      </c>
       <c r="D67" s="8">
-        <v>46162.20453821759</v>
+        <v>46209.797607395834</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>243</v>
@@ -5406,13 +5408,13 @@
         <v>46161</v>
       </c>
       <c r="S67" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U67" s="10" t="s">
-        <v>58</v>
+      <c r="U67" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5487,7 +5489,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46197.59005303241</v>
+        <v>46209.797597094905</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>182</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 22:13 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="289">
   <si>
     <t>50001506 - ZCO EPM FRIO AIRE</t>
   </si>
@@ -4513,9 +4513,11 @@
       <c r="B53" s="8">
         <v>46066.48845478009</v>
       </c>
-      <c r="C53" s="9"/>
+      <c r="C53" s="8">
+        <v>46209.915449293985</v>
+      </c>
       <c r="D53" s="8">
-        <v>46209.78872840278</v>
+        <v>46209.91546185185</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>198</v>
@@ -4549,9 +4551,13 @@
       </c>
       <c r="Q53" s="9"/>
       <c r="R53" s="9"/>
-      <c r="S53" s="9"/>
+      <c r="S53" s="9">
+        <v>1</v>
+      </c>
       <c r="T53" s="9"/>
-      <c r="U53" s="9"/>
+      <c r="U53" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
@@ -4629,7 +4635,7 @@
         <v>46204.594040208336</v>
       </c>
       <c r="D55" s="8">
-        <v>46209.811246377314</v>
+        <v>46209.916215439815</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>206</v>
@@ -4690,9 +4696,11 @@
       <c r="B56" s="5">
         <v>46066.48845053241</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46209.9154271875</v>
+      </c>
       <c r="D56" s="5">
-        <v>46204.59404793981</v>
+        <v>46209.91544646991</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>210</v>
@@ -4737,13 +4745,13 @@
         <v>46126</v>
       </c>
       <c r="S56" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T56" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U56" s="12" t="s">
-        <v>107</v>
+      <c r="U56" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -5170,7 +5178,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46196.59712994213</v>
+        <v>46209.91544568287</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5220,8 +5228,8 @@
       <c r="T64" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="U64" s="10" t="s">
-        <v>58</v>
+      <c r="U64" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-17 20:41 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -157,6 +157,9 @@
     <t>Ingenieria electrica,Revision tableros pruebas</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1213263333570153</t>
   </si>
   <si>
@@ -332,9 +335,6 @@
   </si>
   <si>
     <t>Baja</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213263333570170</t>
@@ -1850,7 +1850,7 @@
         <v>46233.52146950232</v>
       </c>
       <c r="D10" s="5">
-        <v>46233.52148277778</v>
+        <v>46251.62699929398</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1888,13 +1888,13 @@
         <v>1</v>
       </c>
       <c r="T10" s="6"/>
-      <c r="U10" s="11" t="s">
-        <v>33</v>
+      <c r="U10" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8">
         <v>46066.488451296296</v>
@@ -1906,16 +1906,16 @@
         <v>46097.54323589121</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I11" s="8">
         <v>46027</v>
@@ -1939,7 +1939,7 @@
         <v>41</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="Q11" s="8">
         <v>46027</v>
@@ -1959,28 +1959,28 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" s="5">
         <v>46066.48845153935</v>
       </c>
       <c r="C12" s="5">
-        <v>46233.52145454861</v>
+        <v>46251.626983587965</v>
       </c>
       <c r="D12" s="5">
-        <v>46233.521690381946</v>
+        <v>46251.626985254625</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I12" s="5">
         <v>46149</v>
@@ -2001,10 +2001,10 @@
         <v>46</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Q12" s="5">
         <v>46149</v>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" s="8">
         <v>46066.488451770834</v>
@@ -2036,7 +2036,7 @@
         <v>46233.52170266204</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2060,7 +2060,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2077,7 +2077,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46066.48845050926</v>
@@ -2089,7 +2089,7 @@
         <v>46097.54272628472</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2116,13 +2116,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q14" s="5">
         <v>46027</v>
@@ -2142,7 +2142,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B15" s="8">
         <v>46066.48845109953</v>
@@ -2154,7 +2154,7 @@
         <v>46113.56808707176</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2181,13 +2181,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>41</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q15" s="8">
         <v>46027</v>
@@ -2207,7 +2207,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5">
         <v>46066.48845135416</v>
@@ -2219,7 +2219,7 @@
         <v>46114.52533150463</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2246,13 +2246,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>41</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q16" s="5">
         <v>46027</v>
@@ -2272,7 +2272,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B17" s="8">
         <v>46066.48845160879</v>
@@ -2284,7 +2284,7 @@
         <v>46114.525341712964</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
@@ -2311,13 +2311,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="Q17" s="8">
         <v>46027</v>
@@ -2337,7 +2337,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5">
         <v>46066.48845217592</v>
@@ -2349,7 +2349,7 @@
         <v>46167.553930208334</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>25</v>
@@ -2373,7 +2373,7 @@
         <v>26</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>26</v>
@@ -2390,7 +2390,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" s="8">
         <v>46066.48845243055</v>
@@ -2402,7 +2402,7 @@
         <v>46097.542820752315</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
@@ -2429,13 +2429,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q19" s="8">
         <v>46029</v>
@@ -2455,7 +2455,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B20" s="5">
         <v>46066.48845268518</v>
@@ -2467,7 +2467,7 @@
         <v>46114.52558519676</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2494,13 +2494,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="5">
         <v>46036</v>
@@ -2520,7 +2520,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B21" s="8">
         <v>46066.48845292824</v>
@@ -2532,7 +2532,7 @@
         <v>46097.54333050926</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2559,13 +2559,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="Q21" s="8">
         <v>46030</v>
@@ -2585,7 +2585,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B22" s="5">
         <v>46066.488453171296</v>
@@ -2597,16 +2597,16 @@
         <v>46223.81708695602</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I22" s="5">
         <v>46036</v>
@@ -2624,13 +2624,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q22" s="5">
         <v>46036</v>
@@ -2650,7 +2650,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B23" s="8">
         <v>46066.48844994213</v>
@@ -2662,7 +2662,7 @@
         <v>46114.525521250005</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
@@ -2689,13 +2689,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Q23" s="8">
         <v>46036</v>
@@ -2715,7 +2715,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B24" s="5">
         <v>46066.4884502662</v>
@@ -2727,16 +2727,16 @@
         <v>46223.81708303241</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I24" s="5">
         <v>46036</v>
@@ -2754,13 +2754,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q24" s="5">
         <v>46036</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B25" s="8">
         <v>46066.48845053241</v>
@@ -2792,7 +2792,7 @@
         <v>46184.576358645834</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>25</v>
@@ -2816,7 +2816,7 @@
         <v>26</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>26</v>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B26" s="5">
         <v>46066.48845078704</v>
@@ -2843,16 +2843,16 @@
         <v>46128.62625043982</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I26" s="5">
         <v>46038</v>
@@ -2870,13 +2870,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q26" s="5">
         <v>46038</v>
@@ -2888,10 +2888,10 @@
         <v>1</v>
       </c>
       <c r="T26" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U26" s="12" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -2914,10 +2914,10 @@
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I27" s="8">
         <v>46038</v>
@@ -2935,10 +2935,10 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P27" s="9" t="s">
         <v>110</v>
@@ -2949,7 +2949,7 @@
         <v>0</v>
       </c>
       <c r="T27" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U27" s="10" t="s">
         <v>111</v>
@@ -2975,10 +2975,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I28" s="5">
         <v>46042</v>
@@ -2996,7 +2996,7 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>109</v>
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U28" s="10" t="s">
         <v>111</v>
@@ -3036,10 +3036,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I29" s="8">
         <v>46034</v>
@@ -3057,13 +3057,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O29" s="9" t="s">
         <v>117</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q29" s="8">
         <v>46034</v>
@@ -3101,10 +3101,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I30" s="5">
         <v>46034</v>
@@ -3125,7 +3125,7 @@
         <v>116</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>121</v>
@@ -3136,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U30" s="10" t="s">
         <v>111</v>
@@ -3160,10 +3160,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I31" s="8">
         <v>46043</v>
@@ -3195,7 +3195,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U31" s="10" t="s">
         <v>111</v>
@@ -3221,10 +3221,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I32" s="5">
         <v>46041</v>
@@ -3242,13 +3242,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>127</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q32" s="5">
         <v>46038</v>
@@ -3286,10 +3286,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I33" s="8">
         <v>46041</v>
@@ -3310,7 +3310,7 @@
         <v>126</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P33" s="9" t="s">
         <v>130</v>
@@ -3321,7 +3321,7 @@
         <v>0</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U33" s="10" t="s">
         <v>111</v>
@@ -3347,10 +3347,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I34" s="5">
         <v>46042</v>
@@ -3382,7 +3382,7 @@
         <v>0</v>
       </c>
       <c r="T34" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U34" s="10" t="s">
         <v>111</v>
@@ -3408,10 +3408,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I35" s="8">
         <v>46031</v>
@@ -3429,13 +3429,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O35" s="9" t="s">
         <v>136</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q35" s="8">
         <v>46031</v>
@@ -3473,10 +3473,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I36" s="5">
         <v>46031</v>
@@ -3497,7 +3497,7 @@
         <v>135</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>139</v>
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U36" s="10" t="s">
         <v>111</v>
@@ -3534,10 +3534,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I37" s="8">
         <v>46052</v>
@@ -3569,7 +3569,7 @@
         <v>0</v>
       </c>
       <c r="T37" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U37" s="10" t="s">
         <v>111</v>
@@ -3595,10 +3595,10 @@
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I38" s="5">
         <v>46052</v>
@@ -3630,7 +3630,7 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U38" s="10" t="s">
         <v>111</v>
@@ -3677,13 +3677,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>150</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q39" s="8">
         <v>46038</v>
@@ -3745,7 +3745,7 @@
         <v>147</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>153</v>
@@ -3756,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="T40" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U40" s="10" t="s">
         <v>111</v>
@@ -3817,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U41" s="10" t="s">
         <v>111</v>
@@ -3864,13 +3864,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>159</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q42" s="5">
         <v>46038</v>
@@ -3882,7 +3882,7 @@
         <v>1</v>
       </c>
       <c r="T42" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U42" s="10" t="s">
         <v>111</v>
@@ -3932,7 +3932,7 @@
         <v>158</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P43" s="9" t="s">
         <v>162</v>
@@ -3943,7 +3943,7 @@
         <v>0</v>
       </c>
       <c r="T43" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U43" s="10" t="s">
         <v>111</v>
@@ -4004,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U44" s="10" t="s">
         <v>111</v>
@@ -4107,7 +4107,7 @@
         <v>167</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>168</v>
@@ -4852,7 +4852,7 @@
         <v>1</v>
       </c>
       <c r="T58" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U58" s="11" t="s">
         <v>33</v>
@@ -5000,7 +5000,7 @@
         <v>46182.67990290509</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
@@ -5045,10 +5045,10 @@
         <v>0</v>
       </c>
       <c r="T61" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="U61" s="12" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5189,10 +5189,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I64" s="5">
         <v>46127</v>
@@ -5254,10 +5254,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I65" s="8">
         <v>46178</v>
@@ -5319,10 +5319,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I66" s="5">
         <v>46156</v>
@@ -5384,10 +5384,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I67" s="8">
         <v>46160</v>
@@ -5449,10 +5449,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I68" s="5">
         <v>46162</v>
@@ -5514,10 +5514,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="8">
@@ -5577,10 +5577,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5617,7 +5617,7 @@
         <v>32</v>
       </c>
       <c r="U70" s="12" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5727,7 +5727,7 @@
         <v>32</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5741,7 +5741,7 @@
         <v>46237.554240625</v>
       </c>
       <c r="D73" s="8">
-        <v>46237.55425512731</v>
+        <v>46251.62698818287</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5750,10 +5750,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I73" s="8">
         <v>46188</v>
@@ -5855,7 +5855,7 @@
         <v>32</v>
       </c>
       <c r="U74" s="12" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-18 20:38 UTC
</commit_message>
<xml_diff>
--- a/data/50001506 - ZCO EPM FRIO AIRE.xlsx
+++ b/data/50001506 - ZCO EPM FRIO AIRE.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="969" uniqueCount="282">
   <si>
     <t>50001506 - ZCO EPM FRIO AIRE</t>
   </si>
@@ -824,6 +824,10 @@
   </si>
   <si>
     <t>ot 4221- 4222-4223Despacho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESPACHO PARCIAL. 
+FALTA TABLERO PLC POR COMPONENTE PENDIENTE. </t>
   </si>
   <si>
     <t>Costos,Gestion</t>
@@ -1968,7 +1972,7 @@
         <v>46251.626983587965</v>
       </c>
       <c r="D12" s="5">
-        <v>46251.626985254625</v>
+        <v>46252.606471701394</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>55</v>
@@ -2018,8 +2022,8 @@
       <c r="T12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U12" s="11" t="s">
-        <v>33</v>
+      <c r="U12" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
@@ -4753,9 +4757,11 @@
       <c r="B57" s="8">
         <v>46066.488450902776</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46252.60656390047</v>
+      </c>
       <c r="D57" s="8">
-        <v>46230.9102021875</v>
+        <v>46252.60656517361</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>186</v>
@@ -4789,9 +4795,13 @@
       </c>
       <c r="Q57" s="9"/>
       <c r="R57" s="9"/>
-      <c r="S57" s="9"/>
+      <c r="S57" s="9">
+        <v>1</v>
+      </c>
       <c r="T57" s="9"/>
-      <c r="U57" s="9"/>
+      <c r="U57" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
@@ -4995,9 +5005,11 @@
       <c r="B61" s="8">
         <v>46066.48845202546</v>
       </c>
-      <c r="C61" s="9"/>
+      <c r="C61" s="8">
+        <v>46252.60645265046</v>
+      </c>
       <c r="D61" s="8">
-        <v>46182.67990290509</v>
+        <v>46252.60647239583</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>58</v>
@@ -5042,13 +5054,13 @@
         <v>46147</v>
       </c>
       <c r="S61" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T61" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="U61" s="12" t="s">
-        <v>48</v>
+      <c r="U61" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5629,7 +5641,7 @@
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46237.55424878473</v>
+        <v>46252.60605559028</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>254</v>
@@ -5674,9 +5686,11 @@
       <c r="B72" s="5">
         <v>46066.488453541664</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46252.60602412037</v>
+      </c>
       <c r="D72" s="5">
-        <v>46237.55431125</v>
+        <v>46252.60604236111</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>252</v>
@@ -5721,13 +5735,13 @@
         <v>46184</v>
       </c>
       <c r="S72" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T72" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U72" s="12" t="s">
-        <v>48</v>
+      <c r="U72" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5741,7 +5755,7 @@
         <v>46237.554240625</v>
       </c>
       <c r="D73" s="8">
-        <v>46251.62698818287</v>
+        <v>46252.6060424537</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>261</v>
@@ -5791,8 +5805,8 @@
       <c r="T73" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U73" s="11" t="s">
-        <v>33</v>
+      <c r="U73" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5802,9 +5816,11 @@
       <c r="B74" s="5">
         <v>46066.48845425926</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46252.60604829861</v>
+      </c>
       <c r="D74" s="5">
-        <v>46237.55425744213</v>
+        <v>46252.60606318287</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>265</v>
@@ -5849,13 +5865,13 @@
         <v>46190</v>
       </c>
       <c r="S74" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T74" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U74" s="12" t="s">
-        <v>48</v>
+      <c r="U74" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5867,7 +5883,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46240.719684895834</v>
+        <v>46252.606286180555</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>270</v>
@@ -5891,7 +5907,7 @@
         <v>26</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>26</v>
+        <v>271</v>
       </c>
       <c r="M75" s="9" t="s">
         <v>26</v>
@@ -5903,7 +5919,7 @@
         <v>265</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q75" s="8">
         <v>46191</v>
@@ -5917,13 +5933,13 @@
       <c r="T75" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="U75" s="10" t="s">
-        <v>111</v>
+      <c r="U75" s="12" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B76" s="5">
         <v>46066.488451261575</v>
@@ -5933,7 +5949,7 @@
         <v>46091.6514128125</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>25</v>
@@ -5957,7 +5973,7 @@
         <v>26</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>26</v>
@@ -5970,7 +5986,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B77" s="8">
         <v>46066.4884515625</v>
@@ -5980,16 +5996,16 @@
         <v>46203.19655709491</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I77" s="8">
         <v>46195</v>
@@ -6007,13 +6023,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q77" s="8">
         <v>46192</v>
@@ -6033,7 +6049,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B78" s="5">
         <v>46066.48845186342</v>
@@ -6043,16 +6059,16 @@
         <v>46203.19655721065</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I78" s="5">
         <v>46195</v>
@@ -6070,13 +6086,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>270</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q78" s="5">
         <v>46192</v>

</xml_diff>